<commit_message>
TownHall Production & Experience (pt.1)
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configs/Buildings/Town Hall.xlsx
+++ b/Assets/StreamingAssets/Configs/Buildings/Town Hall.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\IdleProject\Assets\StreamingAssets\Configs\Buildings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14214DF8-F0E7-4E10-928A-538E35E218E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{419F00F3-3921-4951-9C23-D4A77CBF5C72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Experience" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>exp_level</t>
   </si>
@@ -86,12 +86,21 @@
   <si>
     <t>upgrade_shards_cost</t>
   </si>
+  <si>
+    <t>gather_per_click</t>
+  </si>
+  <si>
+    <t>gather_per_auto_click</t>
+  </si>
+  <si>
+    <t>auto_click_interval</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -122,6 +131,14 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -143,7 +160,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -181,24 +198,13 @@
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5639,25 +5645,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="D1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="G1" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H1" s="9"/>
@@ -5681,25 +5687,25 @@
       <c r="Z1" s="9"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A2" s="22">
+      <c r="A2" s="5">
         <v>1</v>
       </c>
-      <c r="B2" s="22">
+      <c r="B2" s="5">
         <v>1</v>
       </c>
-      <c r="C2" s="22">
+      <c r="C2" s="5">
         <v>10</v>
       </c>
-      <c r="D2" s="23">
+      <c r="D2" s="6">
         <v>250</v>
       </c>
-      <c r="E2" s="22">
+      <c r="E2" s="5">
         <v>0</v>
       </c>
-      <c r="F2" s="22">
+      <c r="F2" s="5">
         <v>0</v>
       </c>
-      <c r="G2" s="22">
+      <c r="G2" s="5">
         <v>0</v>
       </c>
       <c r="H2" s="12"/>
@@ -5723,25 +5729,25 @@
       <c r="Z2" s="10"/>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A3" s="22">
+      <c r="A3" s="5">
         <v>2</v>
       </c>
-      <c r="B3" s="22">
+      <c r="B3" s="5">
         <v>3</v>
       </c>
-      <c r="C3" s="22">
+      <c r="C3" s="5">
         <v>200</v>
       </c>
-      <c r="D3" s="23">
+      <c r="D3" s="6">
         <v>0</v>
       </c>
-      <c r="E3" s="22">
+      <c r="E3" s="5">
         <v>0</v>
       </c>
-      <c r="F3" s="22">
+      <c r="F3" s="5">
         <v>0</v>
       </c>
-      <c r="G3" s="22">
+      <c r="G3" s="5">
         <v>0</v>
       </c>
       <c r="H3" s="12"/>
@@ -5765,25 +5771,25 @@
       <c r="Z3" s="10"/>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A4" s="22">
+      <c r="A4" s="5">
         <v>3</v>
       </c>
-      <c r="B4" s="22">
+      <c r="B4" s="5">
         <v>5</v>
       </c>
-      <c r="C4" s="22">
+      <c r="C4" s="5">
         <v>500</v>
       </c>
-      <c r="D4" s="23">
+      <c r="D4" s="6">
         <v>0</v>
       </c>
-      <c r="E4" s="22">
+      <c r="E4" s="5">
         <v>0</v>
       </c>
-      <c r="F4" s="22">
+      <c r="F4" s="5">
         <v>0</v>
       </c>
-      <c r="G4" s="22">
+      <c r="G4" s="5">
         <v>0</v>
       </c>
       <c r="H4" s="12"/>
@@ -5807,25 +5813,25 @@
       <c r="Z4" s="10"/>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A5" s="22">
+      <c r="A5" s="5">
         <v>4</v>
       </c>
-      <c r="B5" s="22">
+      <c r="B5" s="5">
         <v>7</v>
       </c>
-      <c r="C5" s="22">
+      <c r="C5" s="5">
         <v>1000</v>
       </c>
-      <c r="D5" s="23">
+      <c r="D5" s="6">
         <v>0</v>
       </c>
-      <c r="E5" s="22">
+      <c r="E5" s="5">
         <v>0</v>
       </c>
-      <c r="F5" s="22">
+      <c r="F5" s="5">
         <v>0</v>
       </c>
-      <c r="G5" s="22">
+      <c r="G5" s="5">
         <v>0</v>
       </c>
       <c r="H5" s="12"/>
@@ -5849,25 +5855,25 @@
       <c r="Z5" s="10"/>
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A6" s="22">
+      <c r="A6" s="5">
         <v>5</v>
       </c>
-      <c r="B6" s="22">
+      <c r="B6" s="5">
         <v>8</v>
       </c>
-      <c r="C6" s="22">
+      <c r="C6" s="5">
         <v>1000</v>
       </c>
-      <c r="D6" s="23">
+      <c r="D6" s="6">
         <v>0</v>
       </c>
-      <c r="E6" s="22">
+      <c r="E6" s="5">
         <v>0</v>
       </c>
-      <c r="F6" s="22">
+      <c r="F6" s="5">
         <v>0</v>
       </c>
-      <c r="G6" s="22">
+      <c r="G6" s="5">
         <v>0</v>
       </c>
       <c r="H6" s="12"/>
@@ -61768,14 +61774,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A1" s="17"/>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
+      <c r="A1" s="18"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
       <c r="I1" s="14"/>
       <c r="J1" s="14"/>
       <c r="K1" s="14"/>
@@ -61796,8 +61802,8 @@
       <c r="Z1" s="14"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A2" s="18"/>
-      <c r="B2" s="18"/>
+      <c r="A2" s="19"/>
+      <c r="B2" s="19"/>
       <c r="C2" s="15"/>
       <c r="D2" s="15"/>
       <c r="E2" s="15"/>
@@ -66871,14 +66877,14 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.88671875" customWidth="1"/>
     <col min="2" max="2" width="15.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>3</v>
       </c>
@@ -66886,7 +66892,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>5</v>
       </c>
@@ -66894,7 +66900,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
         <v>6</v>
       </c>
@@ -66902,7 +66908,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
         <v>7</v>
       </c>
@@ -66910,7 +66916,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
         <v>8</v>
       </c>
@@ -66918,6 +66924,30 @@
         <v>1</v>
       </c>
     </row>
+    <row r="6" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="16">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="17">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>